<commit_message>
Remove stray root db/rebuild, era-accurate NFL team codes, tidy gamesData comments
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_1996_Results.xlsx
+++ b/DBs/nfl/Results/NFL_1996_Results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\TracerProjects2\NFL_Elo\Results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\nfl\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{570E8E87-8F1D-4C9E-B36A-DDC789F4BA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB9DAC69-221A-4903-AE16-25B502E9FCF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{08222BAE-29A9-4715-8469-D43E3BF66812}"/>
   </bookViews>
@@ -97,9 +97,6 @@
     <t>KC</t>
   </si>
   <si>
-    <t>TEN</t>
-  </si>
-  <si>
     <t>PHI</t>
   </si>
   <si>
@@ -170,6 +167,9 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>HOO</t>
   </si>
 </sst>
 </file>
@@ -1386,7 +1386,7 @@
         <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G12" t="s">
         <v>15</v>
@@ -1415,7 +1415,7 @@
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F13" t="s">
         <v>24</v>
@@ -1447,10 +1447,10 @@
         <v>11</v>
       </c>
       <c r="E14" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" t="s">
         <v>26</v>
-      </c>
-      <c r="F14" t="s">
-        <v>27</v>
       </c>
       <c r="G14" t="s">
         <v>15</v>
@@ -1479,10 +1479,10 @@
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G15" t="s">
         <v>14</v>
@@ -1511,10 +1511,10 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" t="s">
         <v>28</v>
-      </c>
-      <c r="F16" t="s">
-        <v>29</v>
       </c>
       <c r="G16" t="s">
         <v>14</v>
@@ -1543,10 +1543,10 @@
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G17" t="s">
         <v>15</v>
@@ -1575,10 +1575,10 @@
         <v>11</v>
       </c>
       <c r="E18" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" t="s">
         <v>30</v>
-      </c>
-      <c r="F18" t="s">
-        <v>31</v>
       </c>
       <c r="G18" t="s">
         <v>14</v>
@@ -1607,10 +1607,10 @@
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G19" t="s">
         <v>15</v>
@@ -1639,10 +1639,10 @@
         <v>11</v>
       </c>
       <c r="E20" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" t="s">
         <v>32</v>
-      </c>
-      <c r="F20" t="s">
-        <v>33</v>
       </c>
       <c r="G20" t="s">
         <v>15</v>
@@ -1671,10 +1671,10 @@
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G21" t="s">
         <v>14</v>
@@ -1703,10 +1703,10 @@
         <v>11</v>
       </c>
       <c r="E22" t="s">
+        <v>33</v>
+      </c>
+      <c r="F22" t="s">
         <v>34</v>
-      </c>
-      <c r="F22" t="s">
-        <v>35</v>
       </c>
       <c r="G22" t="s">
         <v>14</v>
@@ -1735,10 +1735,10 @@
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G23" t="s">
         <v>15</v>
@@ -1767,10 +1767,10 @@
         <v>11</v>
       </c>
       <c r="E24" t="s">
+        <v>35</v>
+      </c>
+      <c r="F24" t="s">
         <v>36</v>
-      </c>
-      <c r="F24" t="s">
-        <v>37</v>
       </c>
       <c r="G24" t="s">
         <v>14</v>
@@ -1799,10 +1799,10 @@
         <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G25" t="s">
         <v>15</v>
@@ -1831,10 +1831,10 @@
         <v>11</v>
       </c>
       <c r="E26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" t="s">
         <v>38</v>
-      </c>
-      <c r="F26" t="s">
-        <v>39</v>
       </c>
       <c r="G26" t="s">
         <v>14</v>
@@ -1863,10 +1863,10 @@
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G27" t="s">
         <v>15</v>
@@ -1895,10 +1895,10 @@
         <v>11</v>
       </c>
       <c r="E28" t="s">
+        <v>39</v>
+      </c>
+      <c r="F28" t="s">
         <v>40</v>
-      </c>
-      <c r="F28" t="s">
-        <v>41</v>
       </c>
       <c r="G28" t="s">
         <v>15</v>
@@ -1927,10 +1927,10 @@
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G29" t="s">
         <v>14</v>
@@ -1959,10 +1959,10 @@
         <v>11</v>
       </c>
       <c r="E30" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" t="s">
         <v>42</v>
-      </c>
-      <c r="F30" t="s">
-        <v>43</v>
       </c>
       <c r="G30" t="s">
         <v>14</v>
@@ -1991,10 +1991,10 @@
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G31" t="s">
         <v>15</v>
@@ -2087,10 +2087,10 @@
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G34" t="s">
         <v>14</v>
@@ -2119,10 +2119,10 @@
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F35" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G35" t="s">
         <v>15</v>
@@ -2154,7 +2154,7 @@
         <v>12</v>
       </c>
       <c r="F36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G36" t="s">
         <v>15</v>
@@ -2183,7 +2183,7 @@
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F37" t="s">
         <v>12</v>
@@ -2215,10 +2215,10 @@
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G38" t="s">
         <v>14</v>
@@ -2247,10 +2247,10 @@
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F39" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G39" t="s">
         <v>15</v>
@@ -2282,7 +2282,7 @@
         <v>18</v>
       </c>
       <c r="F40" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G40" t="s">
         <v>15</v>
@@ -2311,7 +2311,7 @@
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F41" t="s">
         <v>18</v>
@@ -2346,7 +2346,7 @@
         <v>21</v>
       </c>
       <c r="F42" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G42" t="s">
         <v>14</v>
@@ -2375,7 +2375,7 @@
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F43" t="s">
         <v>21</v>
@@ -2407,7 +2407,7 @@
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F44" t="s">
         <v>22</v>
@@ -2442,7 +2442,7 @@
         <v>22</v>
       </c>
       <c r="F45" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G45" t="s">
         <v>14</v>
@@ -2474,7 +2474,7 @@
         <v>24</v>
       </c>
       <c r="F46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G46" t="s">
         <v>14</v>
@@ -2503,7 +2503,7 @@
         <v>11</v>
       </c>
       <c r="E47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F47" t="s">
         <v>24</v>
@@ -2538,7 +2538,7 @@
         <v>23</v>
       </c>
       <c r="F48" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G48" t="s">
         <v>14</v>
@@ -2567,7 +2567,7 @@
         <v>11</v>
       </c>
       <c r="E49" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F49" t="s">
         <v>23</v>
@@ -2599,7 +2599,7 @@
         <v>11</v>
       </c>
       <c r="E50" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F50" t="s">
         <v>17</v>
@@ -2634,7 +2634,7 @@
         <v>17</v>
       </c>
       <c r="F51" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G51" t="s">
         <v>15</v>
@@ -2663,10 +2663,10 @@
         <v>11</v>
       </c>
       <c r="E52" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F52" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G52" t="s">
         <v>14</v>
@@ -2695,10 +2695,10 @@
         <v>11</v>
       </c>
       <c r="E53" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F53" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G53" t="s">
         <v>15</v>
@@ -2727,10 +2727,10 @@
         <v>11</v>
       </c>
       <c r="E54" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F54" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G54" t="s">
         <v>15</v>
@@ -2759,10 +2759,10 @@
         <v>11</v>
       </c>
       <c r="E55" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F55" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G55" t="s">
         <v>14</v>
@@ -2791,7 +2791,7 @@
         <v>11</v>
       </c>
       <c r="E56" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F56" t="s">
         <v>16</v>
@@ -2826,7 +2826,7 @@
         <v>16</v>
       </c>
       <c r="F57" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G57" t="s">
         <v>15</v>
@@ -2855,7 +2855,7 @@
         <v>11</v>
       </c>
       <c r="E58" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F58" t="s">
         <v>19</v>
@@ -2890,7 +2890,7 @@
         <v>19</v>
       </c>
       <c r="F59" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G59" t="s">
         <v>14</v>
@@ -2919,10 +2919,10 @@
         <v>11</v>
       </c>
       <c r="E60" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F60" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G60" t="s">
         <v>14</v>
@@ -2951,10 +2951,10 @@
         <v>11</v>
       </c>
       <c r="E61" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F61" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G61" t="s">
         <v>15</v>
@@ -2986,7 +2986,7 @@
         <v>20</v>
       </c>
       <c r="F62" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G62" t="s">
         <v>15</v>
@@ -3015,7 +3015,7 @@
         <v>11</v>
       </c>
       <c r="E63" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F63" t="s">
         <v>20</v>
@@ -3050,7 +3050,7 @@
         <v>17</v>
       </c>
       <c r="F64" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G64" t="s">
         <v>14</v>
@@ -3079,7 +3079,7 @@
         <v>11</v>
       </c>
       <c r="E65" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F65" t="s">
         <v>17</v>
@@ -3111,7 +3111,7 @@
         <v>11</v>
       </c>
       <c r="E66" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F66" t="s">
         <v>19</v>
@@ -3146,7 +3146,7 @@
         <v>19</v>
       </c>
       <c r="F67" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G67" t="s">
         <v>15</v>
@@ -3175,7 +3175,7 @@
         <v>11</v>
       </c>
       <c r="E68" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F68" t="s">
         <v>21</v>
@@ -3210,7 +3210,7 @@
         <v>21</v>
       </c>
       <c r="F69" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G69" t="s">
         <v>15</v>
@@ -3239,10 +3239,10 @@
         <v>11</v>
       </c>
       <c r="E70" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F70" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G70" t="s">
         <v>14</v>
@@ -3271,10 +3271,10 @@
         <v>11</v>
       </c>
       <c r="E71" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F71" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G71" t="s">
         <v>15</v>
@@ -3303,10 +3303,10 @@
         <v>11</v>
       </c>
       <c r="E72" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F72" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G72" t="s">
         <v>14</v>
@@ -3335,10 +3335,10 @@
         <v>11</v>
       </c>
       <c r="E73" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F73" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G73" t="s">
         <v>15</v>
@@ -3367,10 +3367,10 @@
         <v>11</v>
       </c>
       <c r="E74" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F74" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G74" t="s">
         <v>14</v>
@@ -3399,10 +3399,10 @@
         <v>11</v>
       </c>
       <c r="E75" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F75" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G75" t="s">
         <v>15</v>
@@ -3434,7 +3434,7 @@
         <v>18</v>
       </c>
       <c r="F76" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G76" t="s">
         <v>15</v>
@@ -3463,7 +3463,7 @@
         <v>11</v>
       </c>
       <c r="E77" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F77" t="s">
         <v>18</v>
@@ -3495,7 +3495,7 @@
         <v>11</v>
       </c>
       <c r="E78" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F78" t="s">
         <v>22</v>
@@ -3530,7 +3530,7 @@
         <v>22</v>
       </c>
       <c r="F79" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G79" t="s">
         <v>15</v>
@@ -3562,7 +3562,7 @@
         <v>24</v>
       </c>
       <c r="F80" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G80" t="s">
         <v>15</v>
@@ -3591,7 +3591,7 @@
         <v>11</v>
       </c>
       <c r="E81" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F81" t="s">
         <v>24</v>
@@ -3623,10 +3623,10 @@
         <v>11</v>
       </c>
       <c r="E82" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F82" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G82" t="s">
         <v>15</v>
@@ -3655,10 +3655,10 @@
         <v>11</v>
       </c>
       <c r="E83" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F83" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G83" t="s">
         <v>14</v>
@@ -3687,10 +3687,10 @@
         <v>11</v>
       </c>
       <c r="E84" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F84" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G84" t="s">
         <v>14</v>
@@ -3719,10 +3719,10 @@
         <v>11</v>
       </c>
       <c r="E85" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F85" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G85" t="s">
         <v>15</v>
@@ -3754,7 +3754,7 @@
         <v>23</v>
       </c>
       <c r="F86" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G86" t="s">
         <v>14</v>
@@ -3783,7 +3783,7 @@
         <v>11</v>
       </c>
       <c r="E87" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F87" t="s">
         <v>23</v>
@@ -3818,7 +3818,7 @@
         <v>12</v>
       </c>
       <c r="F88" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G88" t="s">
         <v>14</v>
@@ -3847,7 +3847,7 @@
         <v>11</v>
       </c>
       <c r="E89" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F89" t="s">
         <v>12</v>
@@ -3879,7 +3879,7 @@
         <v>11</v>
       </c>
       <c r="E90" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F90" t="s">
         <v>16</v>
@@ -3914,7 +3914,7 @@
         <v>16</v>
       </c>
       <c r="F91" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G91" t="s">
         <v>14</v>
@@ -3946,7 +3946,7 @@
         <v>19</v>
       </c>
       <c r="F92" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G92" t="s">
         <v>15</v>
@@ -3975,7 +3975,7 @@
         <v>11</v>
       </c>
       <c r="E93" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F93" t="s">
         <v>19</v>
@@ -4010,7 +4010,7 @@
         <v>24</v>
       </c>
       <c r="F94" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G94" t="s">
         <v>14</v>
@@ -4039,7 +4039,7 @@
         <v>11</v>
       </c>
       <c r="E95" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F95" t="s">
         <v>24</v>
@@ -4074,7 +4074,7 @@
         <v>20</v>
       </c>
       <c r="F96" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G96" t="s">
         <v>14</v>
@@ -4103,7 +4103,7 @@
         <v>11</v>
       </c>
       <c r="E97" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F97" t="s">
         <v>20</v>
@@ -4135,7 +4135,7 @@
         <v>11</v>
       </c>
       <c r="E98" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F98" t="s">
         <v>22</v>
@@ -4170,7 +4170,7 @@
         <v>22</v>
       </c>
       <c r="F99" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G99" t="s">
         <v>15</v>
@@ -4199,10 +4199,10 @@
         <v>11</v>
       </c>
       <c r="E100" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F100" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G100" t="s">
         <v>15</v>
@@ -4231,10 +4231,10 @@
         <v>11</v>
       </c>
       <c r="E101" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F101" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G101" t="s">
         <v>14</v>
@@ -4263,10 +4263,10 @@
         <v>11</v>
       </c>
       <c r="E102" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F102" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G102" t="s">
         <v>14</v>
@@ -4295,10 +4295,10 @@
         <v>11</v>
       </c>
       <c r="E103" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F103" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G103" t="s">
         <v>15</v>
@@ -4330,7 +4330,7 @@
         <v>21</v>
       </c>
       <c r="F104" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G104" t="s">
         <v>14</v>
@@ -4359,7 +4359,7 @@
         <v>11</v>
       </c>
       <c r="E105" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F105" t="s">
         <v>21</v>
@@ -4391,10 +4391,10 @@
         <v>11</v>
       </c>
       <c r="E106" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F106" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G106" t="s">
         <v>15</v>
@@ -4423,10 +4423,10 @@
         <v>11</v>
       </c>
       <c r="E107" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F107" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G107" t="s">
         <v>14</v>
@@ -4455,10 +4455,10 @@
         <v>11</v>
       </c>
       <c r="E108" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F108" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G108" t="s">
         <v>15</v>
@@ -4487,10 +4487,10 @@
         <v>11</v>
       </c>
       <c r="E109" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F109" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G109" t="s">
         <v>14</v>
@@ -4519,7 +4519,7 @@
         <v>11</v>
       </c>
       <c r="E110" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F110" t="s">
         <v>13</v>
@@ -4554,7 +4554,7 @@
         <v>13</v>
       </c>
       <c r="F111" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G111" t="s">
         <v>14</v>
@@ -4586,7 +4586,7 @@
         <v>18</v>
       </c>
       <c r="F112" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G112" t="s">
         <v>14</v>
@@ -4615,7 +4615,7 @@
         <v>11</v>
       </c>
       <c r="E113" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F113" t="s">
         <v>18</v>
@@ -4711,7 +4711,7 @@
         <v>11</v>
       </c>
       <c r="E116" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F116" t="s">
         <v>17</v>
@@ -4746,7 +4746,7 @@
         <v>17</v>
       </c>
       <c r="F117" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G117" t="s">
         <v>14</v>
@@ -4778,7 +4778,7 @@
         <v>23</v>
       </c>
       <c r="F118" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G118" t="s">
         <v>14</v>
@@ -4807,7 +4807,7 @@
         <v>11</v>
       </c>
       <c r="E119" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F119" t="s">
         <v>23</v>
@@ -4839,10 +4839,10 @@
         <v>11</v>
       </c>
       <c r="E120" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F120" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G120" t="s">
         <v>14</v>
@@ -4871,10 +4871,10 @@
         <v>11</v>
       </c>
       <c r="E121" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F121" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G121" t="s">
         <v>15</v>
@@ -4906,7 +4906,7 @@
         <v>21</v>
       </c>
       <c r="F122" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G122" t="s">
         <v>15</v>
@@ -4935,7 +4935,7 @@
         <v>11</v>
       </c>
       <c r="E123" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F123" t="s">
         <v>21</v>
@@ -4967,7 +4967,7 @@
         <v>11</v>
       </c>
       <c r="E124" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F124" t="s">
         <v>20</v>
@@ -5002,7 +5002,7 @@
         <v>20</v>
       </c>
       <c r="F125" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G125" t="s">
         <v>15</v>
@@ -5031,10 +5031,10 @@
         <v>11</v>
       </c>
       <c r="E126" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F126" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G126" t="s">
         <v>14</v>
@@ -5063,10 +5063,10 @@
         <v>11</v>
       </c>
       <c r="E127" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F127" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G127" t="s">
         <v>15</v>
@@ -5095,7 +5095,7 @@
         <v>11</v>
       </c>
       <c r="E128" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F128" t="s">
         <v>13</v>
@@ -5130,7 +5130,7 @@
         <v>13</v>
       </c>
       <c r="F129" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G129" t="s">
         <v>15</v>
@@ -5223,10 +5223,10 @@
         <v>11</v>
       </c>
       <c r="E132" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F132" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G132" t="s">
         <v>15</v>
@@ -5255,10 +5255,10 @@
         <v>11</v>
       </c>
       <c r="E133" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F133" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G133" t="s">
         <v>14</v>
@@ -5287,7 +5287,7 @@
         <v>11</v>
       </c>
       <c r="E134" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F134" t="s">
         <v>24</v>
@@ -5322,7 +5322,7 @@
         <v>24</v>
       </c>
       <c r="F135" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G135" t="s">
         <v>15</v>
@@ -5351,10 +5351,10 @@
         <v>11</v>
       </c>
       <c r="E136" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F136" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G136" t="s">
         <v>14</v>
@@ -5383,10 +5383,10 @@
         <v>11</v>
       </c>
       <c r="E137" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F137" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G137" t="s">
         <v>15</v>
@@ -5415,10 +5415,10 @@
         <v>11</v>
       </c>
       <c r="E138" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F138" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G138" t="s">
         <v>15</v>
@@ -5447,10 +5447,10 @@
         <v>11</v>
       </c>
       <c r="E139" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F139" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G139" t="s">
         <v>14</v>
@@ -5607,10 +5607,10 @@
         <v>11</v>
       </c>
       <c r="E144" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F144" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G144" t="s">
         <v>15</v>
@@ -5639,10 +5639,10 @@
         <v>11</v>
       </c>
       <c r="E145" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F145" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G145" t="s">
         <v>14</v>
@@ -5671,10 +5671,10 @@
         <v>11</v>
       </c>
       <c r="E146" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F146" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G146" t="s">
         <v>15</v>
@@ -5703,10 +5703,10 @@
         <v>11</v>
       </c>
       <c r="E147" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F147" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G147" t="s">
         <v>14</v>
@@ -5735,10 +5735,10 @@
         <v>11</v>
       </c>
       <c r="E148" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F148" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G148" t="s">
         <v>15</v>
@@ -5767,10 +5767,10 @@
         <v>11</v>
       </c>
       <c r="E149" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F149" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G149" t="s">
         <v>14</v>
@@ -5799,10 +5799,10 @@
         <v>11</v>
       </c>
       <c r="E150" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F150" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G150" t="s">
         <v>15</v>
@@ -5831,10 +5831,10 @@
         <v>11</v>
       </c>
       <c r="E151" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F151" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G151" t="s">
         <v>14</v>
@@ -5863,7 +5863,7 @@
         <v>11</v>
       </c>
       <c r="E152" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F152" t="s">
         <v>18</v>
@@ -5898,7 +5898,7 @@
         <v>18</v>
       </c>
       <c r="F153" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G153" t="s">
         <v>15</v>
@@ -5927,7 +5927,7 @@
         <v>11</v>
       </c>
       <c r="E154" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F154" t="s">
         <v>16</v>
@@ -5962,7 +5962,7 @@
         <v>16</v>
       </c>
       <c r="F155" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G155" t="s">
         <v>14</v>
@@ -5991,10 +5991,10 @@
         <v>11</v>
       </c>
       <c r="E156" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F156" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G156" t="s">
         <v>14</v>
@@ -6023,10 +6023,10 @@
         <v>11</v>
       </c>
       <c r="E157" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F157" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G157" t="s">
         <v>15</v>
@@ -6055,7 +6055,7 @@
         <v>11</v>
       </c>
       <c r="E158" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F158" t="s">
         <v>22</v>
@@ -6090,7 +6090,7 @@
         <v>22</v>
       </c>
       <c r="F159" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G159" t="s">
         <v>15</v>
@@ -6119,7 +6119,7 @@
         <v>11</v>
       </c>
       <c r="E160" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F160" t="s">
         <v>17</v>
@@ -6154,7 +6154,7 @@
         <v>17</v>
       </c>
       <c r="F161" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G161" t="s">
         <v>14</v>
@@ -6247,7 +6247,7 @@
         <v>11</v>
       </c>
       <c r="E164" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F164" t="s">
         <v>13</v>
@@ -6282,7 +6282,7 @@
         <v>13</v>
       </c>
       <c r="F165" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G165" t="s">
         <v>14</v>
@@ -6311,10 +6311,10 @@
         <v>11</v>
       </c>
       <c r="E166" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F166" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G166" t="s">
         <v>15</v>
@@ -6343,10 +6343,10 @@
         <v>11</v>
       </c>
       <c r="E167" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F167" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G167" t="s">
         <v>14</v>
@@ -6503,7 +6503,7 @@
         <v>11</v>
       </c>
       <c r="E172" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F172" t="s">
         <v>19</v>
@@ -6538,7 +6538,7 @@
         <v>19</v>
       </c>
       <c r="F173" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G173" t="s">
         <v>15</v>
@@ -6567,10 +6567,10 @@
         <v>11</v>
       </c>
       <c r="E174" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F174" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G174" t="s">
         <v>15</v>
@@ -6599,10 +6599,10 @@
         <v>11</v>
       </c>
       <c r="E175" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F175" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G175" t="s">
         <v>14</v>
@@ -6631,10 +6631,10 @@
         <v>11</v>
       </c>
       <c r="E176" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F176" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G176" t="s">
         <v>14</v>
@@ -6663,10 +6663,10 @@
         <v>11</v>
       </c>
       <c r="E177" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F177" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G177" t="s">
         <v>15</v>
@@ -6698,7 +6698,7 @@
         <v>22</v>
       </c>
       <c r="F178" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G178" t="s">
         <v>14</v>
@@ -6727,7 +6727,7 @@
         <v>11</v>
       </c>
       <c r="E179" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F179" t="s">
         <v>22</v>
@@ -6759,7 +6759,7 @@
         <v>11</v>
       </c>
       <c r="E180" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F180" t="s">
         <v>20</v>
@@ -6794,7 +6794,7 @@
         <v>20</v>
       </c>
       <c r="F181" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G181" t="s">
         <v>15</v>
@@ -6823,10 +6823,10 @@
         <v>11</v>
       </c>
       <c r="E182" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F182" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G182" t="s">
         <v>15</v>
@@ -6855,10 +6855,10 @@
         <v>11</v>
       </c>
       <c r="E183" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F183" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G183" t="s">
         <v>14</v>
@@ -6887,7 +6887,7 @@
         <v>11</v>
       </c>
       <c r="E184" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F184" t="s">
         <v>21</v>
@@ -6922,7 +6922,7 @@
         <v>21</v>
       </c>
       <c r="F185" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G185" t="s">
         <v>15</v>
@@ -6954,7 +6954,7 @@
         <v>18</v>
       </c>
       <c r="F186" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G186" t="s">
         <v>14</v>
@@ -6983,7 +6983,7 @@
         <v>11</v>
       </c>
       <c r="E187" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F187" t="s">
         <v>18</v>
@@ -7015,10 +7015,10 @@
         <v>11</v>
       </c>
       <c r="E188" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F188" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G188" t="s">
         <v>14</v>
@@ -7047,10 +7047,10 @@
         <v>11</v>
       </c>
       <c r="E189" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F189" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G189" t="s">
         <v>15</v>
@@ -7082,7 +7082,7 @@
         <v>24</v>
       </c>
       <c r="F190" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G190" t="s">
         <v>14</v>
@@ -7111,7 +7111,7 @@
         <v>11</v>
       </c>
       <c r="E191" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F191" t="s">
         <v>24</v>
@@ -7143,7 +7143,7 @@
         <v>11</v>
       </c>
       <c r="E192" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F192" t="s">
         <v>13</v>
@@ -7178,7 +7178,7 @@
         <v>13</v>
       </c>
       <c r="F193" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G193" t="s">
         <v>15</v>
@@ -7210,7 +7210,7 @@
         <v>12</v>
       </c>
       <c r="F194" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G194" t="s">
         <v>14</v>
@@ -7239,7 +7239,7 @@
         <v>11</v>
       </c>
       <c r="E195" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F195" t="s">
         <v>12</v>
@@ -7271,7 +7271,7 @@
         <v>11</v>
       </c>
       <c r="E196" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F196" t="s">
         <v>18</v>
@@ -7306,7 +7306,7 @@
         <v>18</v>
       </c>
       <c r="F197" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G197" t="s">
         <v>14</v>
@@ -7335,10 +7335,10 @@
         <v>11</v>
       </c>
       <c r="E198" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F198" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G198" t="s">
         <v>14</v>
@@ -7367,10 +7367,10 @@
         <v>11</v>
       </c>
       <c r="E199" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F199" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G199" t="s">
         <v>15</v>
@@ -7399,10 +7399,10 @@
         <v>11</v>
       </c>
       <c r="E200" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F200" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G200" t="s">
         <v>14</v>
@@ -7431,10 +7431,10 @@
         <v>11</v>
       </c>
       <c r="E201" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F201" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G201" t="s">
         <v>15</v>
@@ -7463,10 +7463,10 @@
         <v>11</v>
       </c>
       <c r="E202" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F202" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G202" t="s">
         <v>15</v>
@@ -7495,10 +7495,10 @@
         <v>11</v>
       </c>
       <c r="E203" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F203" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G203" t="s">
         <v>14</v>
@@ -7527,7 +7527,7 @@
         <v>11</v>
       </c>
       <c r="E204" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F204" t="s">
         <v>17</v>
@@ -7562,7 +7562,7 @@
         <v>17</v>
       </c>
       <c r="F205" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G205" t="s">
         <v>15</v>
@@ -7594,7 +7594,7 @@
         <v>19</v>
       </c>
       <c r="F206" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G206" t="s">
         <v>14</v>
@@ -7623,7 +7623,7 @@
         <v>11</v>
       </c>
       <c r="E207" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F207" t="s">
         <v>19</v>
@@ -7655,10 +7655,10 @@
         <v>11</v>
       </c>
       <c r="E208" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F208" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G208" t="s">
         <v>14</v>
@@ -7687,10 +7687,10 @@
         <v>11</v>
       </c>
       <c r="E209" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F209" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G209" t="s">
         <v>15</v>
@@ -7719,7 +7719,7 @@
         <v>11</v>
       </c>
       <c r="E210" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F210" t="s">
         <v>23</v>
@@ -7754,7 +7754,7 @@
         <v>23</v>
       </c>
       <c r="F211" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G211" t="s">
         <v>15</v>
@@ -7847,10 +7847,10 @@
         <v>11</v>
       </c>
       <c r="E214" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F214" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G214" t="s">
         <v>15</v>
@@ -7879,10 +7879,10 @@
         <v>11</v>
       </c>
       <c r="E215" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F215" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G215" t="s">
         <v>14</v>
@@ -7975,7 +7975,7 @@
         <v>11</v>
       </c>
       <c r="E218" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F218" t="s">
         <v>12</v>
@@ -8010,7 +8010,7 @@
         <v>12</v>
       </c>
       <c r="F219" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G219" t="s">
         <v>15</v>
@@ -8103,7 +8103,7 @@
         <v>11</v>
       </c>
       <c r="E222" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F222" t="s">
         <v>18</v>
@@ -8138,7 +8138,7 @@
         <v>18</v>
       </c>
       <c r="F223" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G223" t="s">
         <v>15</v>
@@ -8167,7 +8167,7 @@
         <v>11</v>
       </c>
       <c r="E224" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F224" t="s">
         <v>21</v>
@@ -8202,7 +8202,7 @@
         <v>21</v>
       </c>
       <c r="F225" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G225" t="s">
         <v>14</v>
@@ -8231,10 +8231,10 @@
         <v>11</v>
       </c>
       <c r="E226" t="s">
+        <v>31</v>
+      </c>
+      <c r="F226" t="s">
         <v>32</v>
-      </c>
-      <c r="F226" t="s">
-        <v>33</v>
       </c>
       <c r="G226" t="s">
         <v>14</v>
@@ -8263,10 +8263,10 @@
         <v>11</v>
       </c>
       <c r="E227" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F227" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G227" t="s">
         <v>15</v>
@@ -8295,10 +8295,10 @@
         <v>11</v>
       </c>
       <c r="E228" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F228" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G228" t="s">
         <v>15</v>
@@ -8327,10 +8327,10 @@
         <v>11</v>
       </c>
       <c r="E229" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F229" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G229" t="s">
         <v>14</v>
@@ -8359,7 +8359,7 @@
         <v>11</v>
       </c>
       <c r="E230" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F230" t="s">
         <v>16</v>
@@ -8394,7 +8394,7 @@
         <v>16</v>
       </c>
       <c r="F231" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G231" t="s">
         <v>15</v>
@@ -8423,7 +8423,7 @@
         <v>11</v>
       </c>
       <c r="E232" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F232" t="s">
         <v>19</v>
@@ -8458,7 +8458,7 @@
         <v>19</v>
       </c>
       <c r="F233" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G233" t="s">
         <v>14</v>
@@ -8487,10 +8487,10 @@
         <v>11</v>
       </c>
       <c r="E234" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F234" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G234" t="s">
         <v>15</v>
@@ -8519,10 +8519,10 @@
         <v>11</v>
       </c>
       <c r="E235" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F235" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G235" t="s">
         <v>14</v>
@@ -8551,7 +8551,7 @@
         <v>11</v>
       </c>
       <c r="E236" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F236" t="s">
         <v>24</v>
@@ -8586,7 +8586,7 @@
         <v>24</v>
       </c>
       <c r="F237" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G237" t="s">
         <v>15</v>
@@ -8615,10 +8615,10 @@
         <v>11</v>
       </c>
       <c r="E238" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F238" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G238" t="s">
         <v>14</v>
@@ -8647,10 +8647,10 @@
         <v>11</v>
       </c>
       <c r="E239" t="s">
+        <v>37</v>
+      </c>
+      <c r="F239" t="s">
         <v>38</v>
-      </c>
-      <c r="F239" t="s">
-        <v>39</v>
       </c>
       <c r="G239" t="s">
         <v>15</v>
@@ -8679,10 +8679,10 @@
         <v>11</v>
       </c>
       <c r="E240" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F240" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G240" t="s">
         <v>14</v>
@@ -8711,10 +8711,10 @@
         <v>11</v>
       </c>
       <c r="E241" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F241" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G241" t="s">
         <v>15</v>
@@ -8743,7 +8743,7 @@
         <v>11</v>
       </c>
       <c r="E242" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F242" t="s">
         <v>20</v>
@@ -8778,7 +8778,7 @@
         <v>20</v>
       </c>
       <c r="F243" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G243" t="s">
         <v>14</v>
@@ -8871,10 +8871,10 @@
         <v>11</v>
       </c>
       <c r="E246" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F246" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G246" t="s">
         <v>14</v>
@@ -8903,10 +8903,10 @@
         <v>11</v>
       </c>
       <c r="E247" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F247" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G247" t="s">
         <v>15</v>
@@ -8938,7 +8938,7 @@
         <v>17</v>
       </c>
       <c r="F248" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G248" t="s">
         <v>15</v>
@@ -8967,7 +8967,7 @@
         <v>11</v>
       </c>
       <c r="E249" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F249" t="s">
         <v>17</v>
@@ -8999,7 +8999,7 @@
         <v>11</v>
       </c>
       <c r="E250" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F250" t="s">
         <v>18</v>
@@ -9034,7 +9034,7 @@
         <v>18</v>
       </c>
       <c r="F251" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G251" t="s">
         <v>14</v>
@@ -9063,7 +9063,7 @@
         <v>11</v>
       </c>
       <c r="E252" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F252" t="s">
         <v>19</v>
@@ -9098,7 +9098,7 @@
         <v>19</v>
       </c>
       <c r="F253" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G253" t="s">
         <v>15</v>
@@ -9127,10 +9127,10 @@
         <v>11</v>
       </c>
       <c r="E254" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F254" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G254" t="s">
         <v>15</v>
@@ -9159,10 +9159,10 @@
         <v>11</v>
       </c>
       <c r="E255" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F255" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G255" t="s">
         <v>14</v>
@@ -9191,7 +9191,7 @@
         <v>11</v>
       </c>
       <c r="E256" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F256" t="s">
         <v>21</v>
@@ -9226,7 +9226,7 @@
         <v>21</v>
       </c>
       <c r="F257" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G257" t="s">
         <v>15</v>
@@ -9319,10 +9319,10 @@
         <v>11</v>
       </c>
       <c r="E260" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F260" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G260" t="s">
         <v>14</v>
@@ -9351,10 +9351,10 @@
         <v>11</v>
       </c>
       <c r="E261" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F261" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G261" t="s">
         <v>15</v>
@@ -9447,10 +9447,10 @@
         <v>11</v>
       </c>
       <c r="E264" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F264" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G264" t="s">
         <v>14</v>
@@ -9479,10 +9479,10 @@
         <v>11</v>
       </c>
       <c r="E265" t="s">
+        <v>33</v>
+      </c>
+      <c r="F265" t="s">
         <v>34</v>
-      </c>
-      <c r="F265" t="s">
-        <v>35</v>
       </c>
       <c r="G265" t="s">
         <v>15</v>
@@ -9511,10 +9511,10 @@
         <v>11</v>
       </c>
       <c r="E266" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F266" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G266" t="s">
         <v>14</v>
@@ -9543,10 +9543,10 @@
         <v>11</v>
       </c>
       <c r="E267" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F267" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G267" t="s">
         <v>15</v>
@@ -9575,10 +9575,10 @@
         <v>11</v>
       </c>
       <c r="E268" t="s">
+        <v>35</v>
+      </c>
+      <c r="F268" t="s">
         <v>36</v>
-      </c>
-      <c r="F268" t="s">
-        <v>37</v>
       </c>
       <c r="G268" t="s">
         <v>15</v>
@@ -9607,10 +9607,10 @@
         <v>11</v>
       </c>
       <c r="E269" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F269" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G269" t="s">
         <v>14</v>
@@ -9639,10 +9639,10 @@
         <v>11</v>
       </c>
       <c r="E270" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F270" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G270" t="s">
         <v>15</v>
@@ -9671,10 +9671,10 @@
         <v>11</v>
       </c>
       <c r="E271" t="s">
+        <v>28</v>
+      </c>
+      <c r="F271" t="s">
         <v>29</v>
-      </c>
-      <c r="F271" t="s">
-        <v>30</v>
       </c>
       <c r="G271" t="s">
         <v>14</v>
@@ -9767,10 +9767,10 @@
         <v>11</v>
       </c>
       <c r="E274" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F274" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G274" t="s">
         <v>15</v>
@@ -9799,10 +9799,10 @@
         <v>11</v>
       </c>
       <c r="E275" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F275" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G275" t="s">
         <v>14</v>
@@ -9895,7 +9895,7 @@
         <v>11</v>
       </c>
       <c r="E278" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F278" t="s">
         <v>18</v>
@@ -9930,7 +9930,7 @@
         <v>18</v>
       </c>
       <c r="F279" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G279" t="s">
         <v>15</v>
@@ -9962,7 +9962,7 @@
         <v>19</v>
       </c>
       <c r="F280" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G280" t="s">
         <v>15</v>
@@ -9991,7 +9991,7 @@
         <v>11</v>
       </c>
       <c r="E281" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F281" t="s">
         <v>19</v>
@@ -10026,7 +10026,7 @@
         <v>24</v>
       </c>
       <c r="F282" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G282" t="s">
         <v>14</v>
@@ -10055,7 +10055,7 @@
         <v>11</v>
       </c>
       <c r="E283" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F283" t="s">
         <v>24</v>
@@ -10087,10 +10087,10 @@
         <v>11</v>
       </c>
       <c r="E284" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F284" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G284" t="s">
         <v>15</v>
@@ -10119,10 +10119,10 @@
         <v>11</v>
       </c>
       <c r="E285" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F285" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G285" t="s">
         <v>14</v>
@@ -10151,10 +10151,10 @@
         <v>11</v>
       </c>
       <c r="E286" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F286" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G286" t="s">
         <v>15</v>
@@ -10183,10 +10183,10 @@
         <v>11</v>
       </c>
       <c r="E287" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F287" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G287" t="s">
         <v>14</v>
@@ -10215,10 +10215,10 @@
         <v>11</v>
       </c>
       <c r="E288" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F288" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G288" t="s">
         <v>14</v>
@@ -10247,10 +10247,10 @@
         <v>11</v>
       </c>
       <c r="E289" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F289" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G289" t="s">
         <v>15</v>
@@ -10279,10 +10279,10 @@
         <v>11</v>
       </c>
       <c r="E290" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F290" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G290" t="s">
         <v>14</v>
@@ -10311,10 +10311,10 @@
         <v>11</v>
       </c>
       <c r="E291" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F291" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G291" t="s">
         <v>15</v>
@@ -10343,10 +10343,10 @@
         <v>11</v>
       </c>
       <c r="E292" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F292" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G292" t="s">
         <v>15</v>
@@ -10375,10 +10375,10 @@
         <v>11</v>
       </c>
       <c r="E293" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F293" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G293" t="s">
         <v>14</v>
@@ -10410,7 +10410,7 @@
         <v>22</v>
       </c>
       <c r="F294" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G294" t="s">
         <v>14</v>
@@ -10439,7 +10439,7 @@
         <v>11</v>
       </c>
       <c r="E295" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F295" t="s">
         <v>22</v>
@@ -10471,7 +10471,7 @@
         <v>11</v>
       </c>
       <c r="E296" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F296" t="s">
         <v>20</v>
@@ -10506,7 +10506,7 @@
         <v>20</v>
       </c>
       <c r="F297" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G297" t="s">
         <v>15</v>
@@ -10538,7 +10538,7 @@
         <v>12</v>
       </c>
       <c r="F298" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G298" t="s">
         <v>14</v>
@@ -10567,7 +10567,7 @@
         <v>11</v>
       </c>
       <c r="E299" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F299" t="s">
         <v>12</v>
@@ -10599,7 +10599,7 @@
         <v>11</v>
       </c>
       <c r="E300" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F300" t="s">
         <v>21</v>
@@ -10634,7 +10634,7 @@
         <v>21</v>
       </c>
       <c r="F301" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G301" t="s">
         <v>15</v>
@@ -10666,7 +10666,7 @@
         <v>13</v>
       </c>
       <c r="F302" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G302" t="s">
         <v>14</v>
@@ -10695,7 +10695,7 @@
         <v>11</v>
       </c>
       <c r="E303" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F303" t="s">
         <v>13</v>
@@ -10727,7 +10727,7 @@
         <v>11</v>
       </c>
       <c r="E304" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F304" t="s">
         <v>17</v>
@@ -10762,7 +10762,7 @@
         <v>17</v>
       </c>
       <c r="F305" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G305" t="s">
         <v>15</v>
@@ -10858,7 +10858,7 @@
         <v>24</v>
       </c>
       <c r="F308" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G308" t="s">
         <v>14</v>
@@ -10887,7 +10887,7 @@
         <v>11</v>
       </c>
       <c r="E309" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F309" t="s">
         <v>24</v>
@@ -10922,7 +10922,7 @@
         <v>18</v>
       </c>
       <c r="F310" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G310" t="s">
         <v>14</v>
@@ -10951,7 +10951,7 @@
         <v>11</v>
       </c>
       <c r="E311" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F311" t="s">
         <v>18</v>
@@ -10983,10 +10983,10 @@
         <v>11</v>
       </c>
       <c r="E312" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F312" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G312" t="s">
         <v>15</v>
@@ -11015,10 +11015,10 @@
         <v>11</v>
       </c>
       <c r="E313" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F313" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G313" t="s">
         <v>14</v>
@@ -11050,7 +11050,7 @@
         <v>21</v>
       </c>
       <c r="F314" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G314" t="s">
         <v>14</v>
@@ -11079,7 +11079,7 @@
         <v>11</v>
       </c>
       <c r="E315" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F315" t="s">
         <v>21</v>
@@ -11175,10 +11175,10 @@
         <v>11</v>
       </c>
       <c r="E318" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F318" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G318" t="s">
         <v>15</v>
@@ -11207,10 +11207,10 @@
         <v>11</v>
       </c>
       <c r="E319" t="s">
+        <v>25</v>
+      </c>
+      <c r="F319" t="s">
         <v>26</v>
-      </c>
-      <c r="F319" t="s">
-        <v>27</v>
       </c>
       <c r="G319" t="s">
         <v>14</v>
@@ -11242,7 +11242,7 @@
         <v>19</v>
       </c>
       <c r="F320" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G320" t="s">
         <v>14</v>
@@ -11271,7 +11271,7 @@
         <v>11</v>
       </c>
       <c r="E321" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F321" t="s">
         <v>19</v>
@@ -11303,10 +11303,10 @@
         <v>11</v>
       </c>
       <c r="E322" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F322" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G322" t="s">
         <v>15</v>
@@ -11335,10 +11335,10 @@
         <v>11</v>
       </c>
       <c r="E323" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F323" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G323" t="s">
         <v>14</v>
@@ -11367,10 +11367,10 @@
         <v>11</v>
       </c>
       <c r="E324" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F324" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G324" t="s">
         <v>14</v>
@@ -11399,10 +11399,10 @@
         <v>11</v>
       </c>
       <c r="E325" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F325" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G325" t="s">
         <v>15</v>
@@ -11431,10 +11431,10 @@
         <v>11</v>
       </c>
       <c r="E326" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F326" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G326" t="s">
         <v>15</v>
@@ -11463,10 +11463,10 @@
         <v>11</v>
       </c>
       <c r="E327" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F327" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G327" t="s">
         <v>14</v>
@@ -11498,7 +11498,7 @@
         <v>20</v>
       </c>
       <c r="F328" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G328" t="s">
         <v>15</v>
@@ -11527,7 +11527,7 @@
         <v>11</v>
       </c>
       <c r="E329" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F329" t="s">
         <v>20</v>
@@ -11559,10 +11559,10 @@
         <v>11</v>
       </c>
       <c r="E330" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F330" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G330" t="s">
         <v>14</v>
@@ -11591,10 +11591,10 @@
         <v>11</v>
       </c>
       <c r="E331" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F331" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G331" t="s">
         <v>15</v>
@@ -11687,10 +11687,10 @@
         <v>11</v>
       </c>
       <c r="E334" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F334" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G334" t="s">
         <v>14</v>
@@ -11719,10 +11719,10 @@
         <v>11</v>
       </c>
       <c r="E335" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F335" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G335" t="s">
         <v>15</v>
@@ -11754,7 +11754,7 @@
         <v>12</v>
       </c>
       <c r="F336" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G336" t="s">
         <v>15</v>
@@ -11783,7 +11783,7 @@
         <v>11</v>
       </c>
       <c r="E337" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F337" t="s">
         <v>12</v>
@@ -11815,7 +11815,7 @@
         <v>11</v>
       </c>
       <c r="E338" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F338" t="s">
         <v>21</v>
@@ -11850,7 +11850,7 @@
         <v>21</v>
       </c>
       <c r="F339" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G339" t="s">
         <v>15</v>
@@ -11879,7 +11879,7 @@
         <v>11</v>
       </c>
       <c r="E340" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F340" t="s">
         <v>18</v>
@@ -11914,7 +11914,7 @@
         <v>18</v>
       </c>
       <c r="F341" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G341" t="s">
         <v>15</v>
@@ -11943,7 +11943,7 @@
         <v>11</v>
       </c>
       <c r="E342" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F342" t="s">
         <v>20</v>
@@ -11978,7 +11978,7 @@
         <v>20</v>
       </c>
       <c r="F343" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G343" t="s">
         <v>14</v>
@@ -12010,7 +12010,7 @@
         <v>22</v>
       </c>
       <c r="F344" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G344" t="s">
         <v>15</v>
@@ -12039,7 +12039,7 @@
         <v>11</v>
       </c>
       <c r="E345" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F345" t="s">
         <v>22</v>
@@ -12071,7 +12071,7 @@
         <v>11</v>
       </c>
       <c r="E346" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F346" t="s">
         <v>24</v>
@@ -12106,7 +12106,7 @@
         <v>24</v>
       </c>
       <c r="F347" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G347" t="s">
         <v>14</v>
@@ -12135,10 +12135,10 @@
         <v>11</v>
       </c>
       <c r="E348" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F348" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G348" t="s">
         <v>14</v>
@@ -12167,10 +12167,10 @@
         <v>11</v>
       </c>
       <c r="E349" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F349" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G349" t="s">
         <v>15</v>
@@ -12199,10 +12199,10 @@
         <v>11</v>
       </c>
       <c r="E350" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F350" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G350" t="s">
         <v>15</v>
@@ -12231,10 +12231,10 @@
         <v>11</v>
       </c>
       <c r="E351" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F351" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G351" t="s">
         <v>14</v>
@@ -12266,7 +12266,7 @@
         <v>19</v>
       </c>
       <c r="F352" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G352" t="s">
         <v>14</v>
@@ -12295,7 +12295,7 @@
         <v>11</v>
       </c>
       <c r="E353" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F353" t="s">
         <v>19</v>
@@ -12327,10 +12327,10 @@
         <v>11</v>
       </c>
       <c r="E354" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F354" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G354" t="s">
         <v>14</v>
@@ -12359,10 +12359,10 @@
         <v>11</v>
       </c>
       <c r="E355" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F355" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G355" t="s">
         <v>15</v>
@@ -12391,10 +12391,10 @@
         <v>11</v>
       </c>
       <c r="E356" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F356" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G356" t="s">
         <v>15</v>
@@ -12423,10 +12423,10 @@
         <v>11</v>
       </c>
       <c r="E357" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F357" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G357" t="s">
         <v>14</v>
@@ -12455,7 +12455,7 @@
         <v>11</v>
       </c>
       <c r="E358" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F358" t="s">
         <v>16</v>
@@ -12490,7 +12490,7 @@
         <v>16</v>
       </c>
       <c r="F359" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G359" t="s">
         <v>14</v>
@@ -12522,7 +12522,7 @@
         <v>23</v>
       </c>
       <c r="F360" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G360" t="s">
         <v>15</v>
@@ -12551,7 +12551,7 @@
         <v>11</v>
       </c>
       <c r="E361" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F361" t="s">
         <v>23</v>
@@ -12647,10 +12647,10 @@
         <v>11</v>
       </c>
       <c r="E364" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F364" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G364" t="s">
         <v>14</v>
@@ -12679,10 +12679,10 @@
         <v>11</v>
       </c>
       <c r="E365" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F365" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G365" t="s">
         <v>15</v>
@@ -12714,7 +12714,7 @@
         <v>18</v>
       </c>
       <c r="F366" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G366" t="s">
         <v>14</v>
@@ -12743,7 +12743,7 @@
         <v>11</v>
       </c>
       <c r="E367" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F367" t="s">
         <v>18</v>
@@ -12778,7 +12778,7 @@
         <v>12</v>
       </c>
       <c r="F368" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G368" t="s">
         <v>14</v>
@@ -12807,7 +12807,7 @@
         <v>11</v>
       </c>
       <c r="E369" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F369" t="s">
         <v>12</v>
@@ -12839,10 +12839,10 @@
         <v>11</v>
       </c>
       <c r="E370" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F370" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G370" t="s">
         <v>14</v>
@@ -12871,10 +12871,10 @@
         <v>11</v>
       </c>
       <c r="E371" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F371" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G371" t="s">
         <v>15</v>
@@ -13031,10 +13031,10 @@
         <v>11</v>
       </c>
       <c r="E376" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F376" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G376" t="s">
         <v>14</v>
@@ -13063,10 +13063,10 @@
         <v>11</v>
       </c>
       <c r="E377" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F377" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G377" t="s">
         <v>15</v>
@@ -13095,7 +13095,7 @@
         <v>11</v>
       </c>
       <c r="E378" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F378" t="s">
         <v>23</v>
@@ -13130,7 +13130,7 @@
         <v>23</v>
       </c>
       <c r="F379" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G379" t="s">
         <v>15</v>
@@ -13159,10 +13159,10 @@
         <v>11</v>
       </c>
       <c r="E380" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F380" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G380" t="s">
         <v>14</v>
@@ -13191,10 +13191,10 @@
         <v>11</v>
       </c>
       <c r="E381" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F381" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G381" t="s">
         <v>15</v>
@@ -13223,10 +13223,10 @@
         <v>11</v>
       </c>
       <c r="E382" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F382" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G382" t="s">
         <v>14</v>
@@ -13255,10 +13255,10 @@
         <v>11</v>
       </c>
       <c r="E383" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F383" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G383" t="s">
         <v>15</v>
@@ -13290,7 +13290,7 @@
         <v>16</v>
       </c>
       <c r="F384" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G384" t="s">
         <v>15</v>
@@ -13319,7 +13319,7 @@
         <v>11</v>
       </c>
       <c r="E385" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F385" t="s">
         <v>16</v>
@@ -13351,10 +13351,10 @@
         <v>11</v>
       </c>
       <c r="E386" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F386" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G386" t="s">
         <v>15</v>
@@ -13383,10 +13383,10 @@
         <v>11</v>
       </c>
       <c r="E387" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F387" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G387" t="s">
         <v>14</v>
@@ -13415,10 +13415,10 @@
         <v>11</v>
       </c>
       <c r="E388" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F388" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G388" t="s">
         <v>15</v>
@@ -13447,10 +13447,10 @@
         <v>11</v>
       </c>
       <c r="E389" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F389" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G389" t="s">
         <v>14</v>
@@ -13479,7 +13479,7 @@
         <v>11</v>
       </c>
       <c r="E390" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F390" t="s">
         <v>13</v>
@@ -13514,7 +13514,7 @@
         <v>13</v>
       </c>
       <c r="F391" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G391" t="s">
         <v>14</v>
@@ -13546,7 +13546,7 @@
         <v>18</v>
       </c>
       <c r="F392" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G392" t="s">
         <v>14</v>
@@ -13575,7 +13575,7 @@
         <v>11</v>
       </c>
       <c r="E393" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F393" t="s">
         <v>18</v>
@@ -13610,7 +13610,7 @@
         <v>13</v>
       </c>
       <c r="F394" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G394" t="s">
         <v>15</v>
@@ -13639,7 +13639,7 @@
         <v>11</v>
       </c>
       <c r="E395" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F395" t="s">
         <v>13</v>
@@ -13671,7 +13671,7 @@
         <v>11</v>
       </c>
       <c r="E396" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F396" t="s">
         <v>16</v>
@@ -13706,7 +13706,7 @@
         <v>16</v>
       </c>
       <c r="F397" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G397" t="s">
         <v>15</v>
@@ -13738,7 +13738,7 @@
         <v>17</v>
       </c>
       <c r="F398" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G398" t="s">
         <v>14</v>
@@ -13767,7 +13767,7 @@
         <v>11</v>
       </c>
       <c r="E399" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F399" t="s">
         <v>17</v>
@@ -13799,10 +13799,10 @@
         <v>11</v>
       </c>
       <c r="E400" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F400" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G400" t="s">
         <v>14</v>
@@ -13831,10 +13831,10 @@
         <v>11</v>
       </c>
       <c r="E401" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F401" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G401" t="s">
         <v>15</v>
@@ -13866,7 +13866,7 @@
         <v>22</v>
       </c>
       <c r="F402" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G402" t="s">
         <v>15</v>
@@ -13895,7 +13895,7 @@
         <v>11</v>
       </c>
       <c r="E403" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F403" t="s">
         <v>22</v>
@@ -13927,10 +13927,10 @@
         <v>11</v>
       </c>
       <c r="E404" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F404" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G404" t="s">
         <v>15</v>
@@ -13959,10 +13959,10 @@
         <v>11</v>
       </c>
       <c r="E405" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F405" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G405" t="s">
         <v>14</v>
@@ -13994,7 +13994,7 @@
         <v>23</v>
       </c>
       <c r="F406" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G406" t="s">
         <v>14</v>
@@ -14023,7 +14023,7 @@
         <v>11</v>
       </c>
       <c r="E407" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F407" t="s">
         <v>23</v>
@@ -14055,10 +14055,10 @@
         <v>11</v>
       </c>
       <c r="E408" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F408" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G408" t="s">
         <v>14</v>
@@ -14087,10 +14087,10 @@
         <v>11</v>
       </c>
       <c r="E409" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F409" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G409" t="s">
         <v>15</v>
@@ -14119,10 +14119,10 @@
         <v>11</v>
       </c>
       <c r="E410" t="s">
+        <v>38</v>
+      </c>
+      <c r="F410" t="s">
         <v>39</v>
-      </c>
-      <c r="F410" t="s">
-        <v>40</v>
       </c>
       <c r="G410" t="s">
         <v>14</v>
@@ -14151,10 +14151,10 @@
         <v>11</v>
       </c>
       <c r="E411" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F411" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G411" t="s">
         <v>15</v>
@@ -14186,7 +14186,7 @@
         <v>12</v>
       </c>
       <c r="F412" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G412" t="s">
         <v>15</v>
@@ -14215,7 +14215,7 @@
         <v>11</v>
       </c>
       <c r="E413" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F413" t="s">
         <v>12</v>
@@ -14247,7 +14247,7 @@
         <v>11</v>
       </c>
       <c r="E414" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F414" t="s">
         <v>19</v>
@@ -14282,7 +14282,7 @@
         <v>19</v>
       </c>
       <c r="F415" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G415" t="s">
         <v>14</v>
@@ -14311,10 +14311,10 @@
         <v>11</v>
       </c>
       <c r="E416" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F416" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G416" t="s">
         <v>14</v>
@@ -14343,10 +14343,10 @@
         <v>11</v>
       </c>
       <c r="E417" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F417" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G417" t="s">
         <v>15</v>
@@ -14439,7 +14439,7 @@
         <v>11</v>
       </c>
       <c r="E420" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F420" t="s">
         <v>24</v>
@@ -14474,7 +14474,7 @@
         <v>24</v>
       </c>
       <c r="F421" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G421" t="s">
         <v>15</v>
@@ -14503,10 +14503,10 @@
         <v>11</v>
       </c>
       <c r="E422" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F422" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G422" t="s">
         <v>15</v>
@@ -14535,10 +14535,10 @@
         <v>11</v>
       </c>
       <c r="E423" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F423" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G423" t="s">
         <v>14</v>
@@ -14567,10 +14567,10 @@
         <v>11</v>
       </c>
       <c r="E424" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F424" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G424" t="s">
         <v>14</v>
@@ -14599,10 +14599,10 @@
         <v>11</v>
       </c>
       <c r="E425" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F425" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G425" t="s">
         <v>15</v>
@@ -14698,7 +14698,7 @@
         <v>12</v>
       </c>
       <c r="F428" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G428" t="s">
         <v>14</v>
@@ -14727,7 +14727,7 @@
         <v>11</v>
       </c>
       <c r="E429" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F429" t="s">
         <v>12</v>
@@ -14762,7 +14762,7 @@
         <v>17</v>
       </c>
       <c r="F430" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G430" t="s">
         <v>15</v>
@@ -14791,7 +14791,7 @@
         <v>11</v>
       </c>
       <c r="E431" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F431" t="s">
         <v>17</v>
@@ -14823,10 +14823,10 @@
         <v>11</v>
       </c>
       <c r="E432" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F432" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G432" t="s">
         <v>14</v>
@@ -14855,10 +14855,10 @@
         <v>11</v>
       </c>
       <c r="E433" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F433" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G433" t="s">
         <v>15</v>
@@ -14887,7 +14887,7 @@
         <v>11</v>
       </c>
       <c r="E434" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F434" t="s">
         <v>21</v>
@@ -14922,7 +14922,7 @@
         <v>21</v>
       </c>
       <c r="F435" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G435" t="s">
         <v>14</v>
@@ -14954,7 +14954,7 @@
         <v>20</v>
       </c>
       <c r="F436" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G436" t="s">
         <v>14</v>
@@ -14983,7 +14983,7 @@
         <v>11</v>
       </c>
       <c r="E437" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F437" t="s">
         <v>20</v>
@@ -15015,10 +15015,10 @@
         <v>11</v>
       </c>
       <c r="E438" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F438" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G438" t="s">
         <v>15</v>
@@ -15047,10 +15047,10 @@
         <v>11</v>
       </c>
       <c r="E439" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F439" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G439" t="s">
         <v>14</v>
@@ -15079,7 +15079,7 @@
         <v>11</v>
       </c>
       <c r="E440" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F440" t="s">
         <v>23</v>
@@ -15114,7 +15114,7 @@
         <v>23</v>
       </c>
       <c r="F441" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G441" t="s">
         <v>14</v>
@@ -15210,7 +15210,7 @@
         <v>19</v>
       </c>
       <c r="F444" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G444" t="s">
         <v>14</v>
@@ -15239,7 +15239,7 @@
         <v>11</v>
       </c>
       <c r="E445" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F445" t="s">
         <v>19</v>
@@ -15271,10 +15271,10 @@
         <v>11</v>
       </c>
       <c r="E446" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F446" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G446" t="s">
         <v>14</v>
@@ -15303,10 +15303,10 @@
         <v>11</v>
       </c>
       <c r="E447" t="s">
+        <v>28</v>
+      </c>
+      <c r="F447" t="s">
         <v>29</v>
-      </c>
-      <c r="F447" t="s">
-        <v>30</v>
       </c>
       <c r="G447" t="s">
         <v>15</v>
@@ -15338,7 +15338,7 @@
         <v>22</v>
       </c>
       <c r="F448" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G448" t="s">
         <v>14</v>
@@ -15367,7 +15367,7 @@
         <v>11</v>
       </c>
       <c r="E449" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F449" t="s">
         <v>22</v>
@@ -15399,10 +15399,10 @@
         <v>11</v>
       </c>
       <c r="E450" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F450" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G450" t="s">
         <v>14</v>
@@ -15431,10 +15431,10 @@
         <v>11</v>
       </c>
       <c r="E451" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F451" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G451" t="s">
         <v>15</v>
@@ -15463,10 +15463,10 @@
         <v>11</v>
       </c>
       <c r="E452" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F452" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G452" t="s">
         <v>15</v>
@@ -15495,10 +15495,10 @@
         <v>11</v>
       </c>
       <c r="E453" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F453" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G453" t="s">
         <v>14</v>
@@ -15530,7 +15530,7 @@
         <v>16</v>
       </c>
       <c r="F454" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G454" t="s">
         <v>14</v>
@@ -15559,7 +15559,7 @@
         <v>11</v>
       </c>
       <c r="E455" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F455" t="s">
         <v>16</v>
@@ -15655,7 +15655,7 @@
         <v>11</v>
       </c>
       <c r="E458" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F458" t="s">
         <v>24</v>
@@ -15690,7 +15690,7 @@
         <v>24</v>
       </c>
       <c r="F459" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G459" t="s">
         <v>15</v>
@@ -15783,10 +15783,10 @@
         <v>11</v>
       </c>
       <c r="E462" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F462" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G462" t="s">
         <v>14</v>
@@ -15815,10 +15815,10 @@
         <v>11</v>
       </c>
       <c r="E463" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F463" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G463" t="s">
         <v>15</v>
@@ -15911,7 +15911,7 @@
         <v>11</v>
       </c>
       <c r="E466" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F466" t="s">
         <v>19</v>
@@ -15946,7 +15946,7 @@
         <v>19</v>
       </c>
       <c r="F467" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G467" t="s">
         <v>15</v>
@@ -15975,7 +15975,7 @@
         <v>11</v>
       </c>
       <c r="E468" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F468" t="s">
         <v>20</v>
@@ -16010,7 +16010,7 @@
         <v>20</v>
       </c>
       <c r="F469" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G469" t="s">
         <v>15</v>
@@ -16039,10 +16039,10 @@
         <v>11</v>
       </c>
       <c r="E470" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F470" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G470" t="s">
         <v>15</v>
@@ -16071,10 +16071,10 @@
         <v>11</v>
       </c>
       <c r="E471" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F471" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G471" t="s">
         <v>14</v>
@@ -16103,10 +16103,10 @@
         <v>11</v>
       </c>
       <c r="E472" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F472" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G472" t="s">
         <v>15</v>
@@ -16135,10 +16135,10 @@
         <v>11</v>
       </c>
       <c r="E473" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F473" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G473" t="s">
         <v>14</v>
@@ -16167,10 +16167,10 @@
         <v>11</v>
       </c>
       <c r="E474" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F474" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G474" t="s">
         <v>14</v>
@@ -16199,10 +16199,10 @@
         <v>11</v>
       </c>
       <c r="E475" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F475" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G475" t="s">
         <v>15</v>
@@ -16231,10 +16231,10 @@
         <v>11</v>
       </c>
       <c r="E476" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F476" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G476" t="s">
         <v>15</v>
@@ -16263,10 +16263,10 @@
         <v>11</v>
       </c>
       <c r="E477" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F477" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G477" t="s">
         <v>14</v>
@@ -16295,10 +16295,10 @@
         <v>11</v>
       </c>
       <c r="E478" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F478" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G478" t="s">
         <v>14</v>
@@ -16327,10 +16327,10 @@
         <v>11</v>
       </c>
       <c r="E479" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F479" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G479" t="s">
         <v>15</v>
@@ -16359,7 +16359,7 @@
         <v>11</v>
       </c>
       <c r="E480" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F480" t="s">
         <v>21</v>
@@ -16394,7 +16394,7 @@
         <v>21</v>
       </c>
       <c r="F481" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G481" t="s">
         <v>15</v>
@@ -16417,16 +16417,16 @@
         <v>1996</v>
       </c>
       <c r="C482" t="s">
+        <v>43</v>
+      </c>
+      <c r="D482" t="s">
         <v>44</v>
-      </c>
-      <c r="D482" t="s">
-        <v>45</v>
       </c>
       <c r="E482" t="s">
         <v>22</v>
       </c>
       <c r="F482" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G482" t="s">
         <v>15</v>
@@ -16449,13 +16449,13 @@
         <v>1996</v>
       </c>
       <c r="C483" t="s">
+        <v>43</v>
+      </c>
+      <c r="D483" t="s">
         <v>44</v>
       </c>
-      <c r="D483" t="s">
-        <v>45</v>
-      </c>
       <c r="E483" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F483" t="s">
         <v>22</v>
@@ -16481,13 +16481,13 @@
         <v>1996</v>
       </c>
       <c r="C484" t="s">
+        <v>43</v>
+      </c>
+      <c r="D484" t="s">
         <v>44</v>
       </c>
-      <c r="D484" t="s">
-        <v>45</v>
-      </c>
       <c r="E484" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F484" t="s">
         <v>20</v>
@@ -16513,16 +16513,16 @@
         <v>1996</v>
       </c>
       <c r="C485" t="s">
+        <v>43</v>
+      </c>
+      <c r="D485" t="s">
         <v>44</v>
-      </c>
-      <c r="D485" t="s">
-        <v>45</v>
       </c>
       <c r="E485" t="s">
         <v>20</v>
       </c>
       <c r="F485" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G485" t="s">
         <v>15</v>
@@ -16545,10 +16545,10 @@
         <v>1996</v>
       </c>
       <c r="C486" t="s">
+        <v>43</v>
+      </c>
+      <c r="D486" t="s">
         <v>44</v>
-      </c>
-      <c r="D486" t="s">
-        <v>45</v>
       </c>
       <c r="E486" t="s">
         <v>23</v>
@@ -16577,10 +16577,10 @@
         <v>1996</v>
       </c>
       <c r="C487" t="s">
+        <v>43</v>
+      </c>
+      <c r="D487" t="s">
         <v>44</v>
-      </c>
-      <c r="D487" t="s">
-        <v>45</v>
       </c>
       <c r="E487" t="s">
         <v>18</v>
@@ -16609,16 +16609,16 @@
         <v>1996</v>
       </c>
       <c r="C488" t="s">
+        <v>43</v>
+      </c>
+      <c r="D488" t="s">
         <v>44</v>
       </c>
-      <c r="D488" t="s">
-        <v>45</v>
-      </c>
       <c r="E488" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F488" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G488" t="s">
         <v>14</v>
@@ -16641,16 +16641,16 @@
         <v>1996</v>
       </c>
       <c r="C489" t="s">
+        <v>43</v>
+      </c>
+      <c r="D489" t="s">
         <v>44</v>
       </c>
-      <c r="D489" t="s">
-        <v>45</v>
-      </c>
       <c r="E489" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F489" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G489" t="s">
         <v>15</v>
@@ -16673,16 +16673,16 @@
         <v>1996</v>
       </c>
       <c r="C490" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D490" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E490" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F490" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G490" t="s">
         <v>14</v>
@@ -16705,16 +16705,16 @@
         <v>1996</v>
       </c>
       <c r="C491" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D491" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E491" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F491" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G491" t="s">
         <v>15</v>
@@ -16737,16 +16737,16 @@
         <v>1996</v>
       </c>
       <c r="C492" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D492" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E492" t="s">
         <v>22</v>
       </c>
       <c r="F492" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G492" t="s">
         <v>15</v>
@@ -16769,13 +16769,13 @@
         <v>1996</v>
       </c>
       <c r="C493" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D493" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E493" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F493" t="s">
         <v>22</v>
@@ -16801,13 +16801,13 @@
         <v>1996</v>
       </c>
       <c r="C494" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D494" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E494" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F494" t="s">
         <v>23</v>
@@ -16833,16 +16833,16 @@
         <v>1996</v>
       </c>
       <c r="C495" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D495" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E495" t="s">
         <v>23</v>
       </c>
       <c r="F495" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G495" t="s">
         <v>15</v>
@@ -16865,16 +16865,16 @@
         <v>1996</v>
       </c>
       <c r="C496" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D496" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E496" t="s">
         <v>12</v>
       </c>
       <c r="F496" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G496" t="s">
         <v>14</v>
@@ -16897,13 +16897,13 @@
         <v>1996</v>
       </c>
       <c r="C497" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D497" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E497" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F497" t="s">
         <v>12</v>
@@ -16929,13 +16929,13 @@
         <v>1996</v>
       </c>
       <c r="C498" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D498" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E498" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F498" t="s">
         <v>12</v>
@@ -16961,16 +16961,16 @@
         <v>1996</v>
       </c>
       <c r="C499" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D499" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E499" t="s">
         <v>12</v>
       </c>
       <c r="F499" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G499" t="s">
         <v>15</v>
@@ -16993,13 +16993,13 @@
         <v>1996</v>
       </c>
       <c r="C500" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D500" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E500" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F500" t="s">
         <v>22</v>
@@ -17025,16 +17025,16 @@
         <v>1996</v>
       </c>
       <c r="C501" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D501" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E501" t="s">
         <v>22</v>
       </c>
       <c r="F501" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G501" t="s">
         <v>15</v>
@@ -17057,19 +17057,19 @@
         <v>1996</v>
       </c>
       <c r="C502" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D502" t="s">
+        <v>47</v>
+      </c>
+      <c r="E502" t="s">
+        <v>31</v>
+      </c>
+      <c r="F502" t="s">
+        <v>34</v>
+      </c>
+      <c r="G502" t="s">
         <v>48</v>
-      </c>
-      <c r="E502" t="s">
-        <v>32</v>
-      </c>
-      <c r="F502" t="s">
-        <v>35</v>
-      </c>
-      <c r="G502" t="s">
-        <v>49</v>
       </c>
       <c r="H502">
         <v>35</v>
@@ -17089,19 +17089,19 @@
         <v>1996</v>
       </c>
       <c r="C503" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D503" t="s">
+        <v>47</v>
+      </c>
+      <c r="E503" t="s">
+        <v>34</v>
+      </c>
+      <c r="F503" t="s">
+        <v>31</v>
+      </c>
+      <c r="G503" t="s">
         <v>48</v>
-      </c>
-      <c r="E503" t="s">
-        <v>35</v>
-      </c>
-      <c r="F503" t="s">
-        <v>32</v>
-      </c>
-      <c r="G503" t="s">
-        <v>49</v>
       </c>
       <c r="H503">
         <v>21</v>

</xml_diff>